<commit_message>
Remove unsupported MTHFR single-gene test
- Drop the MTHFR row from settings.xlsx (it included none of the 15
  target genes, so the test produced no output)
- Remove MTHFR from the Cancer Panel report's TARGET GENES line
- Delete the orphaned MTHFR comment file
- Update README single-gene reports note
- Regenerate the Target Test Selection figure without MTHFR
</commit_message>
<xml_diff>
--- a/resources/settings.xlsx
+++ b/resources/settings.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P29"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17.4"/>
   <cols>
     <col width="37.69921875" customWidth="1" style="3" min="1" max="1"/>
@@ -1303,7 +1303,7 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t>MTHFR</t>
+          <t>NUDT15</t>
         </is>
       </c>
       <c r="B16" s="0" t="n">
@@ -1337,7 +1337,7 @@
         <v>0</v>
       </c>
       <c r="L16" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16" s="0" t="n">
         <v>0</v>
@@ -1355,7 +1355,7 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t>NUDT15</t>
+          <t>TPMT</t>
         </is>
       </c>
       <c r="B17" s="0" t="n">
@@ -1389,13 +1389,13 @@
         <v>0</v>
       </c>
       <c r="L17" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" s="0" t="n">
         <v>0</v>
       </c>
       <c r="N17" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O17" s="0" t="n">
         <v>0</v>
@@ -1407,7 +1407,7 @@
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t>TPMT</t>
+          <t>UGT1A1</t>
         </is>
       </c>
       <c r="B18" s="0" t="n">
@@ -1447,10 +1447,10 @@
         <v>0</v>
       </c>
       <c r="N18" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O18" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P18" s="0" t="n">
         <v>0</v>
@@ -1459,7 +1459,7 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t>UGT1A1</t>
+          <t>UGT1A1 DPYD</t>
         </is>
       </c>
       <c r="B19" s="0" t="n">
@@ -1487,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K19" s="0" t="n">
         <v>0</v>
@@ -1511,7 +1511,7 @@
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t>UGT1A1 DPYD</t>
+          <t>VKORC1</t>
         </is>
       </c>
       <c r="B20" s="0" t="n">
@@ -1539,7 +1539,7 @@
         <v>0</v>
       </c>
       <c r="J20" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" s="0" t="n">
         <v>0</v>
@@ -1554,16 +1554,16 @@
         <v>0</v>
       </c>
       <c r="O20" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P20" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t>VKORC1</t>
+          <t>NAT2</t>
         </is>
       </c>
       <c r="B21" s="0" t="n">
@@ -1594,7 +1594,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" s="0" t="n">
         <v>0</v>
@@ -1609,72 +1609,72 @@
         <v>0</v>
       </c>
       <c r="P21" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="0" t="inlineStr">
-        <is>
-          <t>NAT2</t>
-        </is>
-      </c>
-      <c r="B22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="L22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="0" t="n">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ABCG2</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ABCG2</t>
+          <t>CYP2B6</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
@@ -1719,14 +1719,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CYP2B6</t>
+          <t>CYP3A4</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>0</v>
       </c>
       <c r="C24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
@@ -1738,7 +1738,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1771,7 +1771,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CYP3A4</t>
+          <t>CYP3A5</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1790,10 +1790,10 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
@@ -1823,7 +1823,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CYP3A5</t>
+          <t>CYP4F2</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1845,10 +1845,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1875,7 +1875,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CYP4F2</t>
+          <t>DPYD</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1900,10 +1900,10 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1927,7 +1927,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DPYD</t>
+          <t>SLCO1B1</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1955,7 +1955,7 @@
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1964,7 +1964,7 @@
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
@@ -1973,58 +1973,6 @@
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>SLCO1B1</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="n">
-        <v>1</v>
-      </c>
-      <c r="N29" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>